<commit_message>
File Updated on 28/08/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A65E7A9A-8A5A-454A-9071-236E8E08B11C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14372987-5ACF-4869-9743-BBC2A2242025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -233,6 +233,9 @@
   </si>
   <si>
     <t>Not productive enough</t>
+  </si>
+  <si>
+    <t>Productive, but not enough</t>
   </si>
 </sst>
 </file>
@@ -1411,26 +1414,50 @@
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A14" s="13"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="14"/>
-      <c r="I14" s="15" t="str">
+      <c r="A14" s="13">
+        <v>46261</v>
+      </c>
+      <c r="B14" s="14">
+        <v>360</v>
+      </c>
+      <c r="C14" s="14">
+        <v>0</v>
+      </c>
+      <c r="D14" s="14">
+        <v>300</v>
+      </c>
+      <c r="E14" s="14">
+        <v>120</v>
+      </c>
+      <c r="F14" s="14">
+        <v>150</v>
+      </c>
+      <c r="G14" s="14">
+        <v>3</v>
+      </c>
+      <c r="H14" s="14">
+        <v>80</v>
+      </c>
+      <c r="I14" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+        <v>1010</v>
+      </c>
+      <c r="J14" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K14" s="16"/>
-      <c r="L14" s="16"/>
-      <c r="M14" s="16"/>
-      <c r="N14" s="17"/>
+        <v>430</v>
+      </c>
+      <c r="K14" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L14" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M14" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N14" s="17" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="13"/>

</xml_diff>

<commit_message>
File updated on 29/08/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14372987-5ACF-4869-9743-BBC2A2242025}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5390A383-00EE-4771-8A34-EB9CCEB7BB96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1460,26 +1460,50 @@
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A15" s="13"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="15" t="str">
+      <c r="A15" s="13">
+        <v>46262</v>
+      </c>
+      <c r="B15" s="14">
+        <v>360</v>
+      </c>
+      <c r="C15" s="14">
+        <v>0</v>
+      </c>
+      <c r="D15" s="14">
+        <v>120</v>
+      </c>
+      <c r="E15" s="14">
+        <v>0</v>
+      </c>
+      <c r="F15" s="14">
+        <v>150</v>
+      </c>
+      <c r="G15" s="14">
+        <v>3</v>
+      </c>
+      <c r="H15" s="14">
+        <v>120</v>
+      </c>
+      <c r="I15" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="15" t="str">
+        <v>750</v>
+      </c>
+      <c r="J15" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K15" s="16"/>
-      <c r="L15" s="16"/>
-      <c r="M15" s="16"/>
-      <c r="N15" s="17"/>
+        <v>690</v>
+      </c>
+      <c r="K15" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L15" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M15" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N15" s="17" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="13"/>

</xml_diff>

<commit_message>
File Updated on 01/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24D58A75-9BA8-43BF-8DFE-89533CF6D13F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B060FAB4-DCCB-43F6-84CF-872AAC38BB3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1598,26 +1598,50 @@
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+      <c r="A18" s="13">
+        <v>46265</v>
+      </c>
+      <c r="B18" s="14">
+        <v>450</v>
+      </c>
+      <c r="C18" s="14">
+        <v>0</v>
+      </c>
+      <c r="D18" s="14">
+        <v>180</v>
+      </c>
+      <c r="E18" s="14">
+        <v>0</v>
+      </c>
+      <c r="F18" s="14">
+        <v>400</v>
+      </c>
+      <c r="G18" s="14">
+        <v>8</v>
+      </c>
+      <c r="H18" s="14">
+        <v>80</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>1110</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="17"/>
+        <v>330</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="13"/>

</xml_diff>

<commit_message>
File Updated on 04/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B060FAB4-DCCB-43F6-84CF-872AAC38BB3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B52434E9-A27A-4006-8449-C96741341033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -235,7 +235,7 @@
     <t>Not productive enough</t>
   </si>
   <si>
-    <t>Prductive, but not efficient</t>
+    <t>Productive, but not efficient</t>
   </si>
 </sst>
 </file>
@@ -1614,21 +1614,21 @@
         <v>0</v>
       </c>
       <c r="F18" s="14">
-        <v>400</v>
+        <v>250</v>
       </c>
       <c r="G18" s="14">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H18" s="14">
         <v>80</v>
       </c>
       <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v>1110</v>
+        <v>960</v>
       </c>
       <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v>330</v>
+        <v>480</v>
       </c>
       <c r="K18" s="16" t="s">
         <v>55</v>
@@ -1644,92 +1644,188 @@
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15" t="str">
+      <c r="A19" s="13">
+        <v>46266</v>
+      </c>
+      <c r="B19" s="14">
+        <v>390</v>
+      </c>
+      <c r="C19" s="14">
+        <v>0</v>
+      </c>
+      <c r="D19" s="14">
+        <v>60</v>
+      </c>
+      <c r="E19" s="14">
+        <v>25</v>
+      </c>
+      <c r="F19" s="14">
+        <v>400</v>
+      </c>
+      <c r="G19" s="14">
+        <v>8</v>
+      </c>
+      <c r="H19" s="14">
+        <v>60</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>935</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="17"/>
+        <v>505</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15" t="str">
+      <c r="A20" s="13">
+        <v>46267</v>
+      </c>
+      <c r="B20" s="14">
+        <v>360</v>
+      </c>
+      <c r="C20" s="14">
+        <v>0</v>
+      </c>
+      <c r="D20" s="14">
+        <v>150</v>
+      </c>
+      <c r="E20" s="14">
+        <v>0</v>
+      </c>
+      <c r="F20" s="14">
+        <v>350</v>
+      </c>
+      <c r="G20" s="14">
+        <v>7</v>
+      </c>
+      <c r="H20" s="14">
+        <v>60</v>
+      </c>
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
+        <v>920</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
-      <c r="N20" s="17"/>
+        <v>520</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N20" s="17" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" s="13"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14"/>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="15" t="str">
+      <c r="A21" s="13">
+        <v>46268</v>
+      </c>
+      <c r="B21" s="14">
+        <v>360</v>
+      </c>
+      <c r="C21" s="14">
+        <v>0</v>
+      </c>
+      <c r="D21" s="14">
+        <v>50</v>
+      </c>
+      <c r="E21" s="14">
+        <v>0</v>
+      </c>
+      <c r="F21" s="14">
+        <v>180</v>
+      </c>
+      <c r="G21" s="14">
+        <v>3</v>
+      </c>
+      <c r="H21" s="14">
+        <v>240</v>
+      </c>
+      <c r="I21" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="15" t="str">
+        <v>830</v>
+      </c>
+      <c r="J21" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K21" s="16"/>
-      <c r="L21" s="16"/>
-      <c r="M21" s="16"/>
-      <c r="N21" s="17"/>
+        <v>610</v>
+      </c>
+      <c r="K21" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L21" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="N21" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A22" s="13"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="15" t="str">
+      <c r="A22" s="13">
+        <v>46269</v>
+      </c>
+      <c r="B22" s="14">
+        <v>390</v>
+      </c>
+      <c r="C22" s="14">
+        <v>0</v>
+      </c>
+      <c r="D22" s="14">
+        <v>0</v>
+      </c>
+      <c r="E22" s="14">
+        <v>0</v>
+      </c>
+      <c r="F22" s="14">
+        <v>200</v>
+      </c>
+      <c r="G22" s="14">
+        <v>4</v>
+      </c>
+      <c r="H22" s="14">
+        <v>150</v>
+      </c>
+      <c r="I22" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="15" t="str">
+        <v>740</v>
+      </c>
+      <c r="J22" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K22" s="16"/>
-      <c r="L22" s="16"/>
-      <c r="M22" s="16"/>
-      <c r="N22" s="17"/>
+        <v>700</v>
+      </c>
+      <c r="K22" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="L22" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="N22" s="17" t="s">
+        <v>62</v>
+      </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="13"/>

</xml_diff>

<commit_message>
File Updated on 05/09/2026
</commit_message>
<xml_diff>
--- a/12605547.xlsx
+++ b/12605547.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Python\Project Data\776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B52434E9-A27A-4006-8449-C96741341033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A9D8CC-B08F-44D6-A9BA-350EACD9031F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="67">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -1827,27 +1827,51 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A23" s="13"/>
-      <c r="B23" s="14"/>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14"/>
-      <c r="F23" s="14"/>
-      <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
-      <c r="I23" s="15" t="str">
+    <row r="23" spans="1:14" ht="30" x14ac:dyDescent="0.25">
+      <c r="A23" s="13">
+        <v>46270</v>
+      </c>
+      <c r="B23" s="14">
+        <v>420</v>
+      </c>
+      <c r="C23" s="14">
+        <v>0</v>
+      </c>
+      <c r="D23" s="14">
+        <v>120</v>
+      </c>
+      <c r="E23" s="14">
+        <v>0</v>
+      </c>
+      <c r="F23" s="14">
+        <v>0</v>
+      </c>
+      <c r="G23" s="14">
+        <v>0</v>
+      </c>
+      <c r="H23" s="14">
+        <v>60</v>
+      </c>
+      <c r="I23" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="15" t="str">
+        <v>600</v>
+      </c>
+      <c r="J23" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K23" s="16"/>
-      <c r="L23" s="16"/>
-      <c r="M23" s="16"/>
-      <c r="N23" s="17"/>
+        <v>840</v>
+      </c>
+      <c r="K23" s="16" t="s">
+        <v>63</v>
+      </c>
+      <c r="L23" s="16" t="s">
+        <v>54</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="N23" s="17" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="13"/>

</xml_diff>